<commit_message>
Remove sheet protection from DB/SESSION sheets for script access
Office Scripts cannot write to protected sheets in Excel for the Web.
Removed SheetProtection from SESSION, USERS_DB, PROJECTS_DB,
ACTIVITIES_DB, and TEAMS_DB. Only README retains protection (read-only).
Sheets remain hidden — visibility is controlled by the login scripts.

https://claude.ai/code/session_018p9yGR1ShsoVtJ2hFqYrUE
</commit_message>
<xml_diff>
--- a/TimeTracking.xlsx
+++ b/TimeTracking.xlsx
@@ -1735,7 +1735,6 @@
       <c r="E2" t="inlineStr"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="D704"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2801,7 +2800,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="D704"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2947,7 +2945,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="D704"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3077,7 +3074,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="D704"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3203,7 +3199,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="D704"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Add RefreshDropdowns script, make project/activity dropdowns dynamic
After editing projects, activities, or teams in the DB sheets, run
RefreshDropdowns.ts to update all dropdown validations across sheets.
Also changed TIME_ENTRY project/activity dropdowns to use INDIRECT
table references so they auto-update from ProjectsTable/ActivitiesTable.

https://claude.ai/code/session_018p9yGR1ShsoVtJ2hFqYrUE
</commit_message>
<xml_diff>
--- a/TimeTracking.xlsx
+++ b/TimeTracking.xlsx
@@ -40349,10 +40349,10 @@
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid Project" error="Select a project from the list" type="list">
-      <formula1>"Website Redesign,API Platform,Mobile App,Data Pipeline,Brand Refresh"</formula1>
+      <formula1>=INDIRECT("ProjectsTable[ProjectName]")</formula1>
     </dataValidation>
     <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid Activity" error="Select an activity from the list" type="list">
-      <formula1>"Development,Design,Testing,Planning,Client Meeting,Admin"</formula1>
+      <formula1>=INDIRECT("ActivitiesTable[ActivityName]")</formula1>
     </dataValidation>
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid Hours" error="Hours must be 1-16" type="whole" operator="between">
       <formula1>1</formula1>

</xml_diff>